<commit_message>
Add a Reveal In Briefing column, and use it to hide Media Ambush
An eighth "living rules set" column for Stages: Reveal In Briefing (Yes/No,
blank = Yes, the old behaviour). A stage set to No no longer names itself
or its opponent in the pre-stage briefing — the player sees a generic
"something is coming" line instead, with the stage's rewards still shown
underneath so they can still weigh what they're risking.

Set to No on ST19 (Media Ambush) only, matching Cameron's playtest
request to keep the ambush a surprise. Every other stage keeps naming
itself, unchanged.

Pasted the column into the master workbook the same way as the other
seven (raw XML zip-surgery on just the Stages sheet, verified against
the rest of the zip byte-for-byte and against openpyxl's cached formula
values elsewhere in the file before replacing the real workbook).
</commit_message>
<xml_diff>
--- a/design/CoP_Starter_Card_Stage_Data.xlsx
+++ b/design/CoP_Starter_Card_Stage_Data.xlsx
@@ -40361,7 +40361,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:AO46"/>
+  <dimension ref="A1:AP46"/>
   <sheetFormatPr defaultColWidth="8.7421875" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.01171875" customWidth="1"/>
@@ -40387,7 +40387,7 @@
     <col min="29" max="29" width="9.953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:42" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>150</v>
       </c>
@@ -40525,6 +40525,11 @@
           <t xml:space="preserve">Reputation Affects Start</t>
         </is>
       </c>
+      <c r="AP1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reveal In Briefing</t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:41" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
@@ -42907,7 +42912,7 @@
         </is>
       </c>
     </row>
-    <row r="20" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>267</v>
       </c>
@@ -43039,6 +43044,11 @@
         </is>
       </c>
       <c r="AO20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AP20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>

</xml_diff>

<commit_message>
Add SH25/26's booster picker and SH01-03's staff-tier bonus layering
SH25/26 ("host a dinner for a player-selected group") now open a real
picker of that item's booster group instead of doing nothing; SH01-03
work at their base level with no staff hired and add the stated bonus
on top once the named staff role reaches the required tier.

Both features share a new TIER:X target (TIER:Party/National/
Constituency), resolved live from each booster's own Tier cell rather
than a fixed ID list, replacing SH01-03's old hardcoded booster lists
and giving SH25/26's picker the same tier grouping for free.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017CtkD8qbkWhfjeHzV7bJcx
</commit_message>
<xml_diff>
--- a/design/CoP_Starter_Card_Stage_Data.xlsx
+++ b/design/CoP_Starter_Card_Stage_Data.xlsx
@@ -10342,7 +10342,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6DBCFC6-E562-474C-8005-C80E8AAC1DE0}">
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:Y30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.84765625" customWidth="1"/>
@@ -10351,7 +10351,7 @@
     <col min="7" max="7" width="20.04296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="68.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" ht="68.25" x14ac:dyDescent="0.2">
       <c r="A1" s="106" t="s">
         <v>2553</v>
       </c>
@@ -10413,8 +10413,58 @@
           <t xml:space="preserve">Purchase Limit</t>
         </is>
       </c>
-    </row>
-    <row r="2" spans="1:15" ht="108" x14ac:dyDescent="0.2">
+      <c r="P1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Player Choice</t>
+        </is>
+      </c>
+      <c r="Q1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 1 Role</t>
+        </is>
+      </c>
+      <c r="R1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 1 Min Tier</t>
+        </is>
+      </c>
+      <c r="S1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 1 Amount</t>
+        </is>
+      </c>
+      <c r="T1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 2 Role</t>
+        </is>
+      </c>
+      <c r="U1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 2 Min Tier</t>
+        </is>
+      </c>
+      <c r="V1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 2 Amount</t>
+        </is>
+      </c>
+      <c r="W1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 3 Role</t>
+        </is>
+      </c>
+      <c r="X1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 3 Min Tier</t>
+        </is>
+      </c>
+      <c r="Y1" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bonus 3 Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="108" x14ac:dyDescent="0.2">
       <c r="A2" s="107" t="s">
         <v>2566</v>
       </c>
@@ -10438,7 +10488,7 @@
       </c>
       <c r="H2" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">BO01|BO02 +1</t>
+          <t xml:space="preserve">TIER:Party +1</t>
         </is>
       </c>
       <c r="I2" s="107" t="inlineStr">
@@ -10459,8 +10509,30 @@
       <c r="O2" s="108">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" ht="108" x14ac:dyDescent="0.2">
+      <c r="Q2" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Policy Research Assistant</t>
+        </is>
+      </c>
+      <c r="R2" s="108">
+        <v>1</v>
+      </c>
+      <c r="S2" s="108">
+        <v>0</v>
+      </c>
+      <c r="T2" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Policy Research Assistant</t>
+        </is>
+      </c>
+      <c r="U2" s="108">
+        <v>2</v>
+      </c>
+      <c r="V2" s="108">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" ht="108" x14ac:dyDescent="0.2">
       <c r="A3" s="107" t="s">
         <v>2571</v>
       </c>
@@ -10484,7 +10556,7 @@
       </c>
       <c r="H3" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">BO05|BO08|BO09|BO10|BO13|BO15|BO16 +2</t>
+          <t xml:space="preserve">TIER:National +2</t>
         </is>
       </c>
       <c r="I3" s="107" t="inlineStr">
@@ -10505,8 +10577,30 @@
       <c r="O3" s="108">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" ht="94.5" x14ac:dyDescent="0.2">
+      <c r="Q3" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media Spokesperson</t>
+        </is>
+      </c>
+      <c r="R3" s="108">
+        <v>1</v>
+      </c>
+      <c r="S3" s="108">
+        <v>0</v>
+      </c>
+      <c r="T3" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media Spokesperson</t>
+        </is>
+      </c>
+      <c r="U3" s="108">
+        <v>2</v>
+      </c>
+      <c r="V3" s="108">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" ht="94.5" x14ac:dyDescent="0.2">
       <c r="A4" s="107" t="s">
         <v>2576</v>
       </c>
@@ -10530,7 +10624,7 @@
       </c>
       <c r="H4" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">BO03|BO04|BO06|BO07|BO11|BO12|BO14 +2</t>
+          <t xml:space="preserve">TIER:Constituency +2</t>
         </is>
       </c>
       <c r="I4" s="107" t="inlineStr">
@@ -10551,8 +10645,30 @@
       <c r="O4" s="108">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="Q4" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">District Representative</t>
+        </is>
+      </c>
+      <c r="R4" s="108">
+        <v>1</v>
+      </c>
+      <c r="S4" s="108">
+        <v>0</v>
+      </c>
+      <c r="T4" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">District Representative</t>
+        </is>
+      </c>
+      <c r="U4" s="108">
+        <v>2</v>
+      </c>
+      <c r="V4" s="108">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A5" s="107" t="s">
         <v>2581</v>
       </c>
@@ -10603,7 +10719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A6" s="107" t="s">
         <v>2584</v>
       </c>
@@ -10654,7 +10770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A7" s="107" t="s">
         <v>2587</v>
       </c>
@@ -10705,7 +10821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:25" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A8" s="107" t="s">
         <v>2590</v>
       </c>
@@ -10756,7 +10872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:25" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A9" s="107" t="s">
         <v>2593</v>
       </c>
@@ -10807,7 +10923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A10" s="107" t="s">
         <v>2596</v>
       </c>
@@ -10845,7 +10961,7 @@
         </is>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A11" s="107" t="s">
         <v>2599</v>
       </c>
@@ -10883,7 +10999,7 @@
         </is>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A12" s="107" t="s">
         <v>2601</v>
       </c>
@@ -10921,7 +11037,7 @@
         </is>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A13" s="107" t="s">
         <v>2604</v>
       </c>
@@ -10959,7 +11075,7 @@
         </is>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:25" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A14" s="107" t="s">
         <v>2606</v>
       </c>
@@ -10997,7 +11113,7 @@
         </is>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:25" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A15" s="107" t="s">
         <v>2608</v>
       </c>
@@ -11035,7 +11151,7 @@
         </is>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A16" s="107" t="s">
         <v>2611</v>
       </c>
@@ -11073,7 +11189,7 @@
         </is>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A17" s="107" t="s">
         <v>2614</v>
       </c>
@@ -11111,7 +11227,7 @@
         </is>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A18" s="107" t="s">
         <v>2617</v>
       </c>
@@ -11149,7 +11265,7 @@
         </is>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:25" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A19" s="107" t="s">
         <v>2620</v>
       </c>
@@ -11187,7 +11303,7 @@
         </is>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:25" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A20" s="107" t="s">
         <v>2623</v>
       </c>
@@ -11225,7 +11341,7 @@
         </is>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A21" s="107" t="s">
         <v>2626</v>
       </c>
@@ -11282,7 +11398,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A22" s="107" t="s">
         <v>2630</v>
       </c>
@@ -11339,7 +11455,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A23" s="107" t="s">
         <v>2634</v>
       </c>
@@ -11396,7 +11512,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A24" s="107" t="s">
         <v>2638</v>
       </c>
@@ -11453,7 +11569,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A25" s="107" t="s">
         <v>2642</v>
       </c>
@@ -11510,7 +11626,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:25" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A26" s="107" t="s">
         <v>2646</v>
       </c>
@@ -11539,7 +11655,7 @@
       </c>
       <c r="J26" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K26" s="107" t="inlineStr">
@@ -11547,8 +11663,18 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
-    </row>
-    <row r="27" spans="1:15" ht="54.75" x14ac:dyDescent="0.2">
+      <c r="H26" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TIER:National +2</t>
+        </is>
+      </c>
+      <c r="P26" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:25" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A27" s="107" t="s">
         <v>2650</v>
       </c>
@@ -11577,7 +11703,7 @@
       </c>
       <c r="J27" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K27" s="107" t="inlineStr">
@@ -11585,8 +11711,18 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
-    </row>
-    <row r="28" spans="1:15" ht="68.25" x14ac:dyDescent="0.2">
+      <c r="H27" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TIER:Constituency +1</t>
+        </is>
+      </c>
+      <c r="P27" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:25" ht="68.25" x14ac:dyDescent="0.2">
       <c r="A28" s="107" t="s">
         <v>2757</v>
       </c>
@@ -11624,7 +11760,7 @@
         </is>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="68.25" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:25" ht="68.25" x14ac:dyDescent="0.2">
       <c r="A29" s="107" t="s">
         <v>2758</v>
       </c>
@@ -11662,7 +11798,7 @@
         </is>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="68.25" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:25" ht="68.25" x14ac:dyDescent="0.2">
       <c r="A30" s="107" t="s">
         <v>2759</v>
       </c>
@@ -27831,7 +27967,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:E250"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.99609375" customWidth="1"/>
@@ -31572,6 +31708,33 @@
       <c r="E250" t="inlineStr">
         <is>
           <t xml:space="preserve">A data-integrity guard, not expected to be seen by a player.</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" spans="1:5">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">item.choose_heading</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item pop-up, Player Choice item, picker heading</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name}  —  choose a group</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shown instead of the ordinary pop-up when the Shop tab's Player Choice cell for this item is Yes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Save and load the run, and choose one of four protagonists
The game now saves itself to the phone after every stage and whenever
something changes in the Office, and picks the run back up on the next
launch. A level left partway through resumes at the start of the stage
it stopped on. A first launch with no save opens a New Game screen with
four protagonists; Office Management has a New game button that asks
before starting over. The four are placeholders: PC01 keeps Hiro of the
Frontier Party, PC02-PC04 are neutral stand-ins with no party. Nine new
Text-tab rows hold the new wording.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017CtkD8qbkWhfjeHzV7bJcx
</commit_message>
<xml_diff>
--- a/design/CoP_Starter_Card_Stage_Data.xlsx
+++ b/design/CoP_Starter_Card_Stage_Data.xlsx
@@ -27967,7 +27967,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:E251"/>
+  <dimension ref="A1:E260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.99609375" customWidth="1"/>
@@ -31735,6 +31735,184 @@
       <c r="E251" t="inlineStr">
         <is>
           <t xml:space="preserve">Shown instead of the ordinary pop-up when the Shop tab's Player Choice cell for this item is Yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" spans="1:5">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">office.resume_level</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Office, Start button, when a saved run stopped partway through a level</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resume level</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takes the player straight back into the level they were playing, at the stage they had reached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" spans="1:5">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">office.new_game</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Office Management, button; and the heading of the warning it opens</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New game</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" spans="1:5">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">office.new_game_warning</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New game, the warning before the run is thrown away</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Starting a new game ends this run. Your standing, cards, staff and items all go back to the start.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" spans="1:5">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">office.new_game_confirm</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New game warning, confirm button</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start over</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" spans="1:5">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">office.new_game_started</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Office report line, after a protagonist is chosen</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A new run begins. Welcome to the Office, {name}.</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" spans="1:5">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">new_game.title</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New Game screen heading</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Choose your legislator</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shown on first launch, and after New game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" spans="1:5">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">new_game.blurb</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New Game screen, line under the heading</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Who are you in Parliament? You play the whole run as the one you choose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" spans="1:5">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">new_game.no_party</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New Game screen, a protagonist with no party set in player.json</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No party yet</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All four protagonists are placeholders until the cast is decided (data/player.json).</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" spans="1:5">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">new_game.choose</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New Game screen, button under each protagonist</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Play as {name}</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show the opponent's next-next move once a card reveals it
C12 Head Count ("Draw 2. Reveal opponent's next intent.") set an
internal flag and nothing ever read it - the reveal had no display at
all. Now a small second line appears under the opponent's own intent
("Then: Guarding 4") once state.next_intent_revealed is true, hidden
otherwise and always hidden in a press conference (there's no pattern
to peek ahead in there).

New Text-tab row (battle.upcoming_intent), added directly to the
workbook's XML rather than through openpyxl, verified the same careful
way as the last few workbook edits - diffed every file inside the
.xlsx (only the Text sheet and the shared strings changed) and a full
cell-by-cell comparison showing exactly the four new cells, nowhere
else.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017CtkD8qbkWhfjeHzV7bJcx
</commit_message>
<xml_diff>
--- a/design/CoP_Starter_Card_Stage_Data.xlsx
+++ b/design/CoP_Starter_Card_Stage_Data.xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7605" uniqueCount="3140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7609" uniqueCount="3144">
   <si>
     <t>Staff ID</t>
   </si>
@@ -9482,6 +9482,18 @@
   </si>
   <si>
     <t>bonus_if_target_segment_ge_30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battle.upcoming_intent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battle - opponent row, shown only after a card reveals the move after next (C12 Head Count)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Then: {intent}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">intent</t>
   </si>
 </sst>
 </file>
@@ -28675,7 +28687,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:E261"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -32280,6 +32292,20 @@
       </c>
       <c r="D260" t="s">
         <v>1193</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5">
+      <c r="A261" t="s">
+        <v>3140</v>
+      </c>
+      <c r="B261" t="s">
+        <v>3141</v>
+      </c>
+      <c r="C261" t="s">
+        <v>3142</v>
+      </c>
+      <c r="D261" t="s">
+        <v>3143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add firing to the Recruitment shop
A filled Staff role can now be fired: a severance (10% of hiring cost by
default, but a real per-candidate column in the workbook's Staff tab now)
is paid from Funds, the role goes vacant and can be filled with a
different candidate right away, and the fired candidate is greyed out
everywhere they'd otherwise be listed, permanently, for the rest of the
run. Nothing already spent or already earned from that hire is refunded
or clawed back. Cameron's decisions on all of this are recorded in
design/proposals/staff_firing.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017CtkD8qbkWhfjeHzV7bJcx
</commit_message>
<xml_diff>
--- a/design/CoP_Starter_Card_Stage_Data.xlsx
+++ b/design/CoP_Starter_Card_Stage_Data.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16903" uniqueCount="4722">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16918" uniqueCount="4737">
   <si>
     <t>Staff ID</t>
   </si>
@@ -14231,6 +14231,51 @@
   </si>
   <si>
     <t xml:space="preserve">buy_card_t3.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firing Cost from Funds (Yen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each role can hold one hire at a time. Hiring, upgrading and firing are all paid from Funds — firing costs a severance, and someone you fire will never work for you again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">office.fire_staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office · Recruitment shop, a filled role's row — button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">office.fire_staff_warning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office · Recruitment shop, the warning before firing someone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firing {name} costs {cost} Yen in severance. They will never work for you again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name, cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">office.fire_staff_confirm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fire warning, confirm button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fire them</t>
+  </si>
+  <si>
+    <t xml:space="preserve">office.staff_fired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office · Recruitment shop, a role's candidate list — someone fired earlier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fired — will not work for you again.</t>
   </si>
 </sst>
 </file>
@@ -17193,7 +17238,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -17206,9 +17251,10 @@
     <col min="10" max="10" width="26" customWidth="1"/>
     <col min="11" max="11" width="34" customWidth="1"/>
     <col min="12" max="12" width="40" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30" customHeight="1">
+    <row r="1" spans="1:13" ht="30" customHeight="1">
       <c r="A1" s="99" t="s">
         <v>0</v>
       </c>
@@ -17245,8 +17291,11 @@
       <c r="L1" s="99" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" s="99" t="s">
+        <v>4722</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="84" t="s">
         <v>11</v>
       </c>
@@ -17283,8 +17332,11 @@
       <c r="L2" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:12">
+      <c r="M2" s="100">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="84" t="s">
         <v>15</v>
       </c>
@@ -17321,8 +17373,11 @@
       <c r="L3" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:12">
+      <c r="M3" s="100">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="84" t="s">
         <v>18</v>
       </c>
@@ -17359,8 +17414,11 @@
       <c r="L4" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="M4" s="100">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="84" t="s">
         <v>20</v>
       </c>
@@ -17397,8 +17455,11 @@
       <c r="L5" s="84" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="6" spans="1:12">
+      <c r="M5" s="100">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="84" t="s">
         <v>24</v>
       </c>
@@ -17435,8 +17496,11 @@
       <c r="L6" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:12">
+      <c r="M6" s="100">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" s="84" t="s">
         <v>26</v>
       </c>
@@ -17473,8 +17537,11 @@
       <c r="L7" s="84" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:12">
+      <c r="M7" s="100">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" s="84" t="s">
         <v>30</v>
       </c>
@@ -17511,8 +17578,11 @@
       <c r="L8" s="84" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:12">
+      <c r="M8" s="100">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" s="84" t="s">
         <v>33</v>
       </c>
@@ -17549,8 +17619,11 @@
       <c r="L9" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="1:12">
+      <c r="M9" s="100">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" s="84" t="s">
         <v>36</v>
       </c>
@@ -17587,8 +17660,11 @@
       <c r="L10" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="11" spans="1:12">
+      <c r="M10" s="100">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" s="84" t="s">
         <v>39</v>
       </c>
@@ -17625,8 +17701,11 @@
       <c r="L11" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="1:12">
+      <c r="M11" s="100">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" s="84" t="s">
         <v>41</v>
       </c>
@@ -17663,8 +17742,11 @@
       <c r="L12" s="84" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="13" spans="1:12">
+      <c r="M12" s="100">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" s="84" t="s">
         <v>45</v>
       </c>
@@ -17701,8 +17783,11 @@
       <c r="L13" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:12">
+      <c r="M13" s="100">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14" s="84" t="s">
         <v>47</v>
       </c>
@@ -17739,8 +17824,11 @@
       <c r="L14" s="84" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="15" spans="1:12">
+      <c r="M14" s="100">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" s="84" t="s">
         <v>50</v>
       </c>
@@ -17777,8 +17865,11 @@
       <c r="L15" s="84" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" spans="1:12">
+      <c r="M15" s="100">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" s="84" t="s">
         <v>53</v>
       </c>
@@ -17815,8 +17906,11 @@
       <c r="L16" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="17" spans="1:12">
+      <c r="M16" s="100">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" s="84" t="s">
         <v>56</v>
       </c>
@@ -17853,8 +17947,11 @@
       <c r="L17" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="18" spans="1:12">
+      <c r="M17" s="100">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" s="84" t="s">
         <v>59</v>
       </c>
@@ -17891,8 +17988,11 @@
       <c r="L18" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="19" spans="1:12">
+      <c r="M18" s="100">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" s="84" t="s">
         <v>61</v>
       </c>
@@ -17929,8 +18029,11 @@
       <c r="L19" s="84" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="20" spans="1:12">
+      <c r="M19" s="100">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
       <c r="A20" s="84" t="s">
         <v>64</v>
       </c>
@@ -17967,8 +18070,11 @@
       <c r="L20" s="101" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="21" spans="1:12">
+      <c r="M20" s="100">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" s="84" t="s">
         <v>66</v>
       </c>
@@ -18005,8 +18111,11 @@
       <c r="L21" s="84" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="22" spans="1:12">
+      <c r="M21" s="100">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
       <c r="A22" s="84" t="s">
         <v>69</v>
       </c>
@@ -18042,6 +18151,9 @@
       </c>
       <c r="L22" s="84" t="s">
         <v>71</v>
+      </c>
+      <c r="M22" s="100">
+        <v>10000</v>
       </c>
     </row>
   </sheetData>
@@ -33424,7 +33536,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:E271"/>
+  <dimension ref="A1:E275"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -36352,7 +36464,7 @@
         <v>2816</v>
       </c>
       <c r="C204" t="s">
-        <v>2817</v>
+        <v>4723</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -37165,6 +37277,53 @@
       </c>
       <c r="C271" t="s">
         <v>3177</v>
+      </c>
+    </row>
+    <row r="272" spans="1:5">
+      <c r="A272" t="s">
+        <v>4724</v>
+      </c>
+      <c r="B272" t="s">
+        <v>4725</v>
+      </c>
+      <c r="C272" t="s">
+        <v>4726</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5">
+      <c r="A273" t="s">
+        <v>4727</v>
+      </c>
+      <c r="B273" t="s">
+        <v>4728</v>
+      </c>
+      <c r="C273" t="s">
+        <v>4729</v>
+      </c>
+      <c r="D273" t="s">
+        <v>4730</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5">
+      <c r="A274" t="s">
+        <v>4731</v>
+      </c>
+      <c r="B274" t="s">
+        <v>4732</v>
+      </c>
+      <c r="C274" t="s">
+        <v>4733</v>
+      </c>
+    </row>
+    <row r="275" spans="1:5">
+      <c r="A275" t="s">
+        <v>4734</v>
+      </c>
+      <c r="B275" t="s">
+        <v>4735</v>
+      </c>
+      <c r="C275" t="s">
+        <v>4736</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove the last of lean_down: its orphaned Text-tab wording
The lean_down committee-chair verb itself was removed from code in
d2d51cb3 (2026-09-24); its wording was deliberately left in the Text tab
at the time as a harmless note. Deleting it now: intent.pressuring,
narration.leaned, narration.lean_none, narration.a_member. Nothing in
scripts/ or tests/ referenced any of the four (confirmed by grep before
removing), so this is wording-only.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017CtkD8qbkWhfjeHzV7bJcx
</commit_message>
<xml_diff>
--- a/design/CoP_Starter_Card_Stage_Data.xlsx
+++ b/design/CoP_Starter_Card_Stage_Data.xlsx
@@ -33937,20 +33937,6 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
-      <c r="A27" t="s">
-        <v>1182</v>
-      </c>
-      <c r="B27" t="s">
-        <v>1169</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>1183</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>1184</v>
-      </c>
-    </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
         <v>1185</v>
@@ -34323,38 +34309,6 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
-      <c r="A52" t="s">
-        <v>1258</v>
-      </c>
-      <c r="B52" t="s">
-        <v>1241</v>
-      </c>
-      <c r="C52" s="13" t="s">
-        <v>1259</v>
-      </c>
-      <c r="D52" t="s">
-        <v>1260</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>1261</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5">
-      <c r="A53" t="s">
-        <v>1262</v>
-      </c>
-      <c r="B53" t="s">
-        <v>1241</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>1263</v>
-      </c>
-      <c r="D53" t="s">
-        <v>1235</v>
-      </c>
-      <c r="E53" s="13"/>
-    </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
         <v>1264</v>
@@ -35916,23 +35870,6 @@
         <v>1210</v>
       </c>
       <c r="E165" s="13"/>
-    </row>
-    <row r="166" spans="1:5">
-      <c r="A166" t="s">
-        <v>1543</v>
-      </c>
-      <c r="B166" t="s">
-        <v>1533</v>
-      </c>
-      <c r="C166" s="13" t="s">
-        <v>1544</v>
-      </c>
-      <c r="D166" t="s">
-        <v>1210</v>
-      </c>
-      <c r="E166" s="13" t="s">
-        <v>1545</v>
-      </c>
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">

</xml_diff>